<commit_message>
#117 write-back 분산락 TrySync
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cshyeon\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6ED62A-E3C0-46E4-B432-2FCFB11CBCB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97294240-5133-4812-B4E6-13F92C8DAE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="ERROR_CODE" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>NONE</t>
   </si>
@@ -83,6 +83,10 @@
   </si>
   <si>
     <t>DISABLED_WHISPER_TARGET</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DISTRIBUTED_LOCK_FAILED</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -481,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.375" style="1" bestFit="1" customWidth="1"/>
@@ -608,6 +612,14 @@
         <v>14</v>
       </c>
     </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: implement clan member position change functionality
- Add ChangeClanPosition API endpoint in ClanController.cs with distributed locks and permission checks
- Add ChangeClanPosition FlatBuffer schema for request/response with host field
- Implement change_clan_member_position method in context with HTTP request
- Add on_clan_change_position AMQP response handler with host filtering
- Add change_position method to clan class for member position updates
- Add builtin_change_position Lua function for clan position changes
- Update error codes to be more specific for clan operations
- Generate FlatBuffer C# and C++ code for new protocol
- Add clan position change functionality to 낙랑 NPC script
- Update clan menu with position change option and proper error handling
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cshyeon\git\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CAAA745-6176-47D5-890C-FDB0D37409B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41A441B-F36A-4A47-A929-AC6E1F52555D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="ERROR_CODE" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>NONE</t>
   </si>
@@ -166,6 +166,18 @@
   </si>
   <si>
     <t>NOT_FOUND_MAIL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>INVALID_CLAN_POSITION</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CANNOT_KICK_SELF</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CANNOT_CHANGE_CLAN_POSITION_SELF</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -232,7 +244,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -564,10 +576,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -859,6 +871,30 @@
         <v>35</v>
       </c>
     </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: implement ban system with reason and expiration date
- Add ban table and repository with soft delete support
- Implement ban/unban API endpoints in internal server
- Add ban check during login and transfer processes
- Add in-game ban/unban commands with operator privileges
- Add AMQP handler for real-time ban notifications
- Add build_ban_message utility function for consistent ban messages
- Change ban_reason from optional string to required string in protocol
- Display ban reason and expiration date to banned users
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C3F366B-DFF6-4767-8809-B70FD178D41E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE6426E-EAD3-4FAD-9060-17F1FC895983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="ERROR_CODE" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>NONE</t>
   </si>
@@ -182,6 +182,13 @@
   </si>
   <si>
     <t>INVALID_CLAN_ROLE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NOT_FOUND_BAN</t>
+  </si>
+  <si>
+    <t>BANNED</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -248,7 +255,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -580,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
@@ -907,6 +914,22 @@
         <v>39</v>
       </c>
     </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add marketplace server
- Create marketplace server with single-database implementation
- Add marketplace API endpoints (list, cancel, purchase, search, check-status, pending)
- Implement marketplace repository with database operations
- Add marketplace service interface for future sharding support
- Add FlatBuffer protocol definitions for marketplace
- Add database schema for marketplace tables
- Remove marketplace design documents
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EE6426E-EAD3-4FAD-9060-17F1FC895983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4238D5-6B93-4DA2-AADC-3EEEB0F53FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="ERROR_CODE" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>NONE</t>
   </si>
@@ -190,6 +190,39 @@
   <si>
     <t>BANNED</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MARKETPLACE_LISTING_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_LISTING_EXPIRED</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_NOT_LISTING_OWNER</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_LISTING_ALREADY_SOLD</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_LISTING_ALREADY_CANCELLED</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_INSUFFICIENT_FUNDS</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_INVALID_PRICE</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_INVALID_EXPIRE_HOURS</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_ITEM_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_PENDING_TRANSACTION_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_PENDING_RETURN_NOT_FOUND</t>
   </si>
 </sst>
 </file>
@@ -255,7 +288,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -587,7 +620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
@@ -930,6 +963,94 @@
         <v>41</v>
       </c>
     </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B45" s="1">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B46" s="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B49" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B50" s="1">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B51" s="1">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52" s="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B53" s="1">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: implement marketplace game server client and remove success field from responses
- Add marketplace.h and marketplace.cpp for game server client
- Implement allocate_id, list, cancel, purchase, search, check_status methods
- Register marketplace request/response types in server.h
- Remove success field from marketplace response protocol (use error field only)
- Update C++ and C# code to use error field for success/failure detection
- Add marketplace.cpp to game.vcxproj
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4238D5-6B93-4DA2-AADC-3EEEB0F53FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2C568C3-CAFC-4FB0-8F0B-46F0552C3E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>NONE</t>
   </si>
@@ -223,6 +223,9 @@
   </si>
   <si>
     <t>MARKETPLACE_PENDING_RETURN_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>MARKETPLACE_INVALID_PAGE_NUMBER</t>
   </si>
 </sst>
 </file>
@@ -620,7 +623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B53"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
@@ -1051,6 +1054,14 @@
         <v>52</v>
       </c>
     </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B54" s="1">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: implement maintenance system
- Add maintenance status check in login and transfer flows
- Add MaintenanceService and MaintenanceCacheService
- Add MaintenanceBackgroundService for scheduled maintenance
- Add admin tool maintenance management page
- Add StartMaintenance protocol message
- Add maintenance message handling in login handler
- Add maintenance error code and messages
- Add Redis lock script for maintenance coordination
- Update protocol definitions for maintenance fields
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9B1CA88-5A7D-4D90-8C04-5F929F394142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A9A627-886B-46CF-ACEF-D08786217889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="ERROR_CODE" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>NONE</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>MARKETPLACE_LISTING_LIMIT_EXCEEDED</t>
+  </si>
+  <si>
+    <t>MAINTENANCE</t>
   </si>
 </sst>
 </file>
@@ -632,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
@@ -1095,6 +1098,14 @@
         <v>56</v>
       </c>
     </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B58" s="1">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add matchmaking table data and model definitions
- Add matchmaking and enum.matchmaking spreadsheet sources
- Regenerate model definitions and enum.error entries
- Update data export script for new tables
</commit_message>
<xml_diff>
--- a/resources/table/enum.error.xlsx
+++ b/resources/table/enum.error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA6A988-08BA-4F63-9FFD-3A21FB750A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44AC18A7-BEC5-4510-805E-BD18998A330E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="ERROR_CODE" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>NONE</t>
   </si>
@@ -242,6 +242,36 @@
   <si>
     <t>MARKETPLACE_ITEM_NOT_TRADEABLE</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MATCHMAKING_UNKNOWN_QUEUE</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_ALREADY_ENROLLED</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_DUPLICATE_ENTRY</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_REGISTRY_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_NOT_PARTICIPANT</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_MATCH_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_ALREADY_CONFIRMED</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_ALREADY_DECLINED</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_CONFIRM_EXPIRED</t>
+  </si>
+  <si>
+    <t>MATCHMAKING_NOT_IN_WAITING_STATE</t>
   </si>
 </sst>
 </file>
@@ -639,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF0AC299-6373-444B-B465-F5D3A155A1B8}">
-  <dimension ref="A1:B59"/>
+  <dimension ref="A1:B69"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" style="1" bestFit="1" customWidth="1"/>
@@ -1118,6 +1148,86 @@
         <v>58</v>
       </c>
     </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B60" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B61" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B62" s="1">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B63" s="1">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B64" s="1">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B65" s="1">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B66" s="1">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B67" s="1">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B68" s="1">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B69" s="1">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>